<commit_message>
Daily jobs update 2026-10-01
</commit_message>
<xml_diff>
--- a/devnetjobs_tracker.xlsx
+++ b/devnetjobs_tracker.xlsx
@@ -556,7 +556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -586,6 +586,19 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-10-01 15:23:31 UTC</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>